<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-03 Les galets de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-03.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le chemin de galets de Nina</t>
+          <t>Les galets de Nina</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, Raphaël, papa, maman</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut un chemin de galets jusqu'à l'escargot. Raphaël reste au banc. Elle répète. Il observe d'abord. Le chemin arrive.</t>
+          <t>Une goutte froide touche le nez de Nina. Sur un galet, un éclat de galet brille. Elle veut un chemin jusqu'à l'escargot, maintenant. Trop de galets d'un coup : ils glissent. Sourire parti. Papa à sa hauteur. Elle répète : un galet, une couleur. Elle regarde d'abord, pose le gris. Merci vécu. Trois galets trop vite : l'éclat manque. Elle refuse de foncer. L'éclat de galet tient sur le bleu.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une gouttière chante encore, tout fin. L'eau tombe dans un seau de zinc. Le seau a un cercle de mousse. Des galets luisent dans la terre noire. On dirait des bonbons mouillés. Tu as vu le seau, Nina ? Il a de la mousse. Tout autour. La pluie l'a laissée. Je veux un chemin. Jusqu'à l'escargot. Un galet après l'autre, alors. L'escargot avance sur une pierre. Très lentement. L'herbe mouillée colle aux chaussures. Ça sent la terre, tout près. Une feuille collée brille sur le banc. Tu as senti la terre ? Oui. Elle est mouillée. En ce moment, Nina est au jardin. Maman essuie le banc avec la main. Le bois reste froid et sombre. Raphaël reste près du banc. Ses mains restent sur le bois mouillé. Raphaël. Tu viens ? Raphaël ne vient pas encore. Il a besoin de calme. Tu peux dire comment on pose. Un galet gris brille près du pied de Nina. L'escargot n'a presque pas bougé.</t>
+          <t>Une goutte froide tombe de la branche. Elle touche le nez de Nina. Oh, c'est froid ! C'est la pluie, dans les feuilles. Un oiseau secoue une feuille, là-haut. La feuille collée brille sur le banc. Tu as vu la feuille, Nina ? Elle brille, maman. Le bois est sombre, dessous. Maman essuie le banc avec la main. Le bois reste froid et sombre. Tu as senti la terre ? Oui, papa. Elle est mouillée. L'herbe mouillée colle aux chaussures. Ça sent la terre, tout près. Tes chaussures sont mouillées. Elles collent, papa. On reste près du banc. D'accord, maman. Des galets luisent dans la terre noire. Sur un galet, un éclat de galet brille. Il brille, papa ! C'est l'eau, sur la pierre. Je veux un chemin, maintenant ! Jusqu'à l'escargot. Un galet. Une couleur. Un escargot avance sur une pierre. Tu as vu l'escargot, Nina ? Il va, maman. On le laisse sur sa pierre. On marche vers les galets ? Oui, papa. Nina a une idée, très nette. Tous les galets, d'un coup ! Nina prend trop de galets, d'un coup. Elle les jette vers la pierre. Les galets glissent dans la boue. Oh. Le chemin ne se fait pas. Le sourire de Nina disparaît. L'éclat de galet tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent, un peu lourdes. Ça tape fort, dans sa poitrine. Papa se met à sa hauteur. Tu veux le chemin ? Oui, papa. En ce moment, Nina pose les mains sur le bois. Ses doigts restent là, sans bouger. Le banc est lisse, un peu froid. Tu restes un peu, Nina ? Oui. Elle regarde l'escargot, sans avancer. L'escargot n'a presque pas bougé.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une gouttière chante encore, tout fin. L'eau tombe dans un seau de zinc. Le seau a un cercle de mousse. Des galets luisent dans la terre noire. On dirait des bonbons mouillés. Tu as vu le seau, Nina ? Il a de la mousse. Tout autour. La pluie l'a laissée. Je veux un chemin. Jusqu'à l'escargot. Un galet après l'autre, alors. L'escargot avance sur une pierre. Très lentement. L'herbe mouillée colle aux chaussures. Ça sent la terre, tout près. Une feuille collée brille sur le banc. Tu as senti la terre ? Oui. Elle est mouillée. En ce moment, Nina est au jardin. Maman essuie le banc avec la main. Le bois reste froid et sombre. Raphaël reste près du banc. Ses mains restent sur le bois mouillé. Raphaël. Tu viens ? Raphaël ne vient pas encore. Il a besoin de calme. Tu peux dire comment on pose. Un galet gris brille près du pied de Nina. L'escargot n'a presque pas bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte froide tombe de la branche. Elle touche le nez de Nina. Oh, c'est froid ! C'est la pluie, dans les feuilles. Un oiseau secoue une feuille, là-haut. La feuille collée brille sur le banc. Tu as vu la feuille, Nina ? Elle brille, maman. Le bois est sombre, dessous. Maman essuie le banc avec la main. Le bois reste froid et sombre. Tu as senti la terre ? Oui, papa. Elle est mouillée. L'herbe mouillée colle aux chaussures. Ça sent la terre, tout près. Tes chaussures sont mouillées. Elles collent, papa. On reste près du banc. D'accord, maman. Des galets luisent dans la terre noire. Sur un galet, un &lt;emphasis level="moderate"&gt;éclat de galet&lt;/emphasis&gt; brille. Il brille, papa ! C'est l'eau, sur la pierre. Je veux un chemin, maintenant ! Jusqu'à l'escargot. Un galet. Une couleur. Un escargot avance sur une pierre. Tu as vu l'escargot, Nina ? Il va, maman. On le laisse sur sa pierre. On marche vers les galets ? Oui, papa. Nina a une idée, très nette. Tous les galets, d'un coup ! Nina prend trop de galets, d'un coup. Elle les jette vers la pierre. Les galets glissent dans la boue. Oh. Le chemin ne se fait pas. Le sourire de Nina disparaît. L'éclat de galet tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent, un peu lourdes. Ça tape fort, dans sa poitrine. Papa se met à sa hauteur. Tu veux le chemin ? Oui, papa. En ce moment, Nina pose les mains sur le bois. Ses doigts restent là, sans bouger. Le banc est lisse, un peu froid. Tu restes un peu, Nina ? Oui. Elle regarde l'escargot, sans avancer. L'escargot n'a presque pas bougé.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sami et Léa sont au jardin avec maman. Maman dit un jeu : on pose un galet. On dit une couleur. Léa reste près du banc. Elle a besoin de calme. Sami va &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. Il dit : un galet, une couleur. Léa écoute. Elle va observer d'abord. Elle regarde. Elle ne joue pas encore. Maman dit : observer d'abord, c'est possible. Sami pose un galet gris. Il dit : gris. Léa sourit. Plus tard, Léa pose un galet aussi. Maman dit : tu as su répéter. Léa a pu observer d'abord. [pause]</t>
+          <t>Une goutte froide tombe de la branche. Elle touche le nez de Nina. Oh, c'est froid ! C'est la pluie, dans les feuilles. Un oiseau secoue une feuille, là-haut. La feuille collée brille sur le banc. Tu as vu la feuille, Nina ? Elle brille, maman. Le bois est sombre, dessous. Maman essuie le banc avec la main. Le bois reste froid et sombre. Tu as senti la terre ? Oui, papa. Elle est mouillée. L'herbe mouillée colle aux chaussures. Ça sent la terre, tout près. Tes chaussures sont mouillées. Elles collent, papa. On reste près du banc. D'accord, maman. Des galets luisent dans la terre noire. Sur un galet, un &lt;emphasis&gt;éclat de galet&lt;/emphasis&gt; brille. Il brille, papa ! C'est l'eau, sur la pierre. Je veux un chemin, maintenant ! Jusqu'à l'escargot. Un galet. Une couleur. Un escargot avance sur une pierre. Tu as vu l'escargot, Nina ? Il va, maman. On le laisse sur sa pierre. On marche vers les galets ? Oui, papa. Nina a une idée, très nette. Tous les galets, d'un coup ! Nina prend trop de galets, d'un coup. Elle les jette vers la pierre. Les galets glissent dans la boue. Oh. Le chemin ne se fait pas. Le sourire de Nina disparaît. L'éclat de galet tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent, un peu lourdes. Ça tape fort, dans sa poitrine. Papa se met à sa hauteur. Tu veux le chemin ? Oui, papa. En ce moment, Nina pose les mains sur le bois. Ses doigts restent là, sans bouger. Le banc est lisse, un peu froid. Tu restes un peu, Nina ? Oui. Elle regarde l'escargot, sans avancer. L'escargot n'a presque pas bougé. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de galet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,46 +1326,75 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_chemin_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une gouttière chante encore, tout fin.
-narrateur|L'eau tombe dans un seau de zinc.
-narrateur|Le seau a un cercle de mousse.
-narrateur|Des galets luisent dans la terre noire.
-narrateur|On dirait des bonbons mouillés.
-maman|Tu as vu le seau, Nina ?
-enfant-f|Il a de la mousse.
-enfant-f|Tout autour.
-maman|La pluie l'a laissée.
-enfant-f|Je veux un chemin.
-enfant-f|Jusqu'à l'escargot.
-maman|Un galet après l'autre, alors.
-narrateur|L'escargot avance sur une pierre.
-narrateur|Très lentement.
+          <t>narrateur|Une goutte froide tombe de la branche.
+narrateur|Elle touche le nez de Nina.
+enfant-f|Oh, c'est froid !
+papa|C'est la pluie, dans les feuilles.
+narrateur|Un oiseau secoue une feuille, là-haut.
+narrateur|La feuille collée brille sur le banc.
+maman|Tu as vu la feuille, Nina ?
+enfant-f|Elle brille, maman.
+maman|Le bois est sombre, dessous.
+narrateur|Maman essuie le banc avec la main.
+narrateur|Le bois reste froid et sombre.
+papa|Tu as senti la terre ?
+enfant-f|Oui, papa.
+enfant-f|Elle est mouillée.
 narrateur|L'herbe mouillée colle aux chaussures.
 narrateur|Ça sent la terre, tout près.
-narrateur|Une feuille collée brille sur le banc.
-maman|Tu as senti la terre ?
+papa|Tes chaussures sont mouillées.
+enfant-f|Elles collent, papa.
+maman|On reste près du banc.
+enfant-f|D'accord, maman.
+narrateur|Des galets luisent dans la terre noire.
+narrateur|Sur un galet, un éclat de galet brille.
+enfant-f|Il brille, papa !
+papa|C'est l'eau, sur la pierre.
+enfant-f|Je veux un chemin, maintenant !
+enfant-f|Jusqu'à l'escargot.
+maman|Un galet.
+maman|Une couleur.
+narrateur|Un escargot avance sur une pierre.
+maman|Tu as vu l'escargot, Nina ?
+enfant-f|Il va, maman.
+maman|On le laisse sur sa pierre.
+papa|On marche vers les galets ?
+enfant-f|Oui, papa.
+narrateur|Nina a une idée, très nette.
+enfant-f|Tous les galets, d'un coup !
+narrateur|Nina prend trop de galets, d'un coup.
+narrateur|Elle les jette vers la pierre.
+narrateur|Les galets glissent dans la boue.
+enfant-f|Oh.
+narrateur|Le chemin ne se fait pas.
+narrateur|Le sourire de Nina disparaît.
+narrateur|L'éclat de galet tremble, puis tient.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Ça ne veut pas.
+narrateur|Ses épaules tombent, un peu lourdes.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Papa se met à sa hauteur.
+papa|Tu veux le chemin ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Nina pose les mains sur le bois.
+narrateur|Ses doigts restent là, sans bouger.
+narrateur|Le banc est lisse, un peu froid.
+papa|Tu restes un peu, Nina ?
 enfant-f|Oui.
-enfant-f|Elle est mouillée.
-narrateur|En ce moment, Nina est au jardin.
-narrateur|Maman essuie le banc avec la main.
-narrateur|Le bois reste froid et sombre.
-narrateur|Raphaël reste près du banc.
-narrateur|Ses mains restent sur le bois mouillé.
-enfant-f|Raphaël.
-enfant-f|Tu viens ?
-narrateur|Raphaël ne vient pas encore.
-maman|Il a besoin de calme.
-maman|Tu peux dire comment on pose.
-narrateur|Un galet gris brille près du pied de Nina.
+narrateur|Elle regarde l'escargot, sans avancer.
 narrateur|L'escargot n'a presque pas bougé.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>gouttiere,jardin</t>
+          <t>jardin,feuilles</t>
         </is>
       </c>
     </row>
@@ -1392,17 +1421,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a besoin de calme. Que peut-on faire ?</t>
+          <t>Nina a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Léa a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1427,7 +1456,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut répéter. On peut observer d'abord. Que fait-on ?</t>
+          <t>On répète. Un galet, une couleur. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1465,18 +1494,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1491,34 +1520,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1527,28 +1560,28 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_a_besoin_de_calme_on_peut_repeter; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a besoin de calme.
+          <t>narrateur|Nina a besoin de calme.
 narrateur|Que peut-on faire ?</t>
         </is>
       </c>
@@ -1576,17 +1609,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina va vers le banc. Elle parle tout doux. On pose un galet. On dit une couleur. Tu as su répéter. Raphaël écoute. Il va observer d'abord. Nina pose un galet gris. Gris. Le galet fait un petit bruit sur la terre. Raphaël suit des yeux. Observer d'abord, c'est possible. Nina pose un galet brun. Brun. Le chemin avance vers la pierre. Plus tard, Raphaël prend un galet bleu. Il le pose, tout doux. Bleu. Bravo, Nina. Tu as laissé le temps. Le dernier galet touche la pierre. L'escargot est encore là. Le chemin est arrivé. Oui. Sans le presser.</t>
+          <t>Papa parle, près du banc. Un galet. Une couleur. Un galet. Une couleur. Nina veut tout prendre, d'un coup. Nina refuse de foncer, cette fois. Elle referme les mains, un instant. Elle regarde les galets, dans la boue. Elle ne prend rien, d'abord. Tu regardes, Nina ? Oui, maman. Elle choisit un galet gris. Gris. Le galet fait un petit bruit sur la terre. Merci, Nina. Papa a vu le gris rester. Sur le gris, l'éclat de galet brille. Il est là. Sur ce gris ? Oui, maman. Nina pose un galet brun, plus loin. Brun. Le chemin avance vers la pierre. Il tient, celui-là ? Oui, papa. L'escargot avance d'un tout petit pas. Il est là, maman. Sur sa pierre ? Oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina va vers le banc. Elle parle tout doux. On pose un galet. On dit une couleur. Tu as su répéter. Raphaël écoute. Il va observer d'abord. Nina pose un galet gris. Gris. Le galet fait un petit bruit sur la terre. Raphaël suit des yeux. Observer d'abord, c'est possible. Nina pose un galet brun. Brun. Le chemin avance vers la pierre. Plus tard, Raphaël prend un galet bleu. Il le pose, tout doux. Bleu. Bravo, Nina. Tu as laissé le temps. Le dernier galet touche la pierre. L'escargot est encore là. Le chemin est arrivé. Oui. Sans le presser.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa parle, près du banc. Un galet. Une couleur. Un galet. Une couleur. Nina veut tout prendre, d'un coup. Nina refuse de foncer, cette fois. Elle referme les mains, un instant. Elle regarde les galets, dans la boue. Elle ne prend rien, d'abord. Tu regardes, Nina ? Oui, maman. Elle choisit un galet gris. Gris. Le galet fait un petit bruit sur la terre. Merci, Nina. Papa a vu le gris rester. Sur le gris, l'&lt;emphasis level="moderate"&gt;éclat de galet&lt;/emphasis&gt; brille. Il est là. Sur ce gris ? Oui, maman. Nina pose un galet brun, plus loin. Brun. Le chemin avance vers la pierre. Il tient, celui-là ? Oui, papa. L'escargot avance d'un tout petit pas. Il est là, maman. Sur sa pierre ? Oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sami a répété. Léa a observé d'abord. Puis elle a joué un peu. [pause]</t>
+          <t>Papa parle, près du banc. Un galet. Une couleur. Un galet. Une couleur. Nina veut tout prendre, d'un coup. Nina refuse de foncer, cette fois. Elle referme les mains, un instant. Elle regarde les galets, dans la boue. Elle ne prend rien, d'abord. Tu regardes, Nina ? Oui, maman. Elle choisit un galet gris. Gris. Le galet fait un petit bruit sur la terre. Merci, Nina. Papa a vu le gris rester. Sur le gris, l'&lt;emphasis&gt;éclat de galet&lt;/emphasis&gt; brille. Il est là. Sur ce gris ? Oui, maman. Nina pose un galet brun, plus loin. Brun. Le chemin avance vers la pierre. Il tient, celui-là ? Oui, papa. L'escargot avance d'un tout petit pas. Il est là, maman. Sur sa pierre ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1633,7 +1666,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1641,10 +1674,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1665,28 +1698,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>éclat de galet</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1695,10 +1732,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1711,36 +1748,41 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_repète_regarde_pose_le_gris; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina va vers le banc.
-narrateur|Elle parle tout doux.
-enfant-f|On pose un galet.
-enfant-f|On dit une couleur.
-maman|Tu as su répéter.
-narrateur|Raphaël écoute.
-narrateur|Il va observer d'abord.
-narrateur|Nina pose un galet gris.
+          <t>narrateur|Papa parle, près du banc.
+papa|Un galet.
+papa|Une couleur.
+enfant-f|Un galet.
+enfant-f|Une couleur.
+narrateur|Nina veut tout prendre, d'un coup.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Elle referme les mains, un instant.
+narrateur|Elle regarde les galets, dans la boue.
+narrateur|Elle ne prend rien, d'abord.
+maman|Tu regardes, Nina ?
+enfant-f|Oui, maman.
+narrateur|Elle choisit un galet gris.
 enfant-f|Gris.
 narrateur|Le galet fait un petit bruit sur la terre.
-narrateur|Raphaël suit des yeux.
-maman|Observer d'abord, c'est possible.
-narrateur|Nina pose un galet brun.
+papa|Merci, Nina.
+narrateur|Papa a vu le gris rester.
+narrateur|Sur le gris, l'éclat de galet brille.
+enfant-f|Il est là.
+maman|Sur ce gris ?
+enfant-f|Oui, maman.
+narrateur|Nina pose un galet brun, plus loin.
 enfant-f|Brun.
 narrateur|Le chemin avance vers la pierre.
-narrateur|Plus tard, Raphaël prend un galet bleu.
-narrateur|Il le pose, tout doux.
-enfant-f|Bleu.
-maman|Bravo, Nina.
-maman|Tu as laissé le temps.
-narrateur|Le dernier galet touche la pierre.
-narrateur|L'escargot est encore là.
-enfant-f|Le chemin est arrivé.
-maman|Oui.
-maman|Sans le presser.</t>
+papa|Il tient, celui-là ?
+enfant-f|Oui, papa.
+narrateur|L'escargot avance d'un tout petit pas.
+enfant-f|Il est là, maman.
+maman|Sur sa pierre ?
+enfant-f|Oui.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1772,17 +1814,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau chante dans l'arbre. J'ai entendu, depuis la cuisine. Vous avez fait un chemin ? Jusqu'à l'escargot. Il est encore sur sa pierre ? Oui, papa. Raphaël a regardé d'abord. Nina a répété la règle. Tu as fini de ranger, Nina ? Oui, maman. Nina donne la main. Raphaël donne l'autre main. Les chaussures laissent des traces mouillées. La gouttière chante plus bas, maintenant. Les galets sont froids. Ils vont sécher. Le seau a encore sa mousse. L'escargot n'a presque pas bougé.</t>
+          <t>Un oiseau chante dans l'arbre. J'ai entendu. Tu as entendu l'oiseau ? Oui, papa. Tout haut. Nina veut arriver, d'un coup. Elle prend trois galets trop vite. Un galet roule vers la pierre. Ça tombe ! L'éclat de galet n'est plus là. Il est parti. Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde les galets, un à un. Elle écoute le jardin, un instant. Comme tout à l'heure ? Tu le vois, toi ? Non, plus sur le gris. Nina cherche près de la pierre. Il est là. Sur ce bleu ? Oui, sur ce galet. Elle pose le bleu, sans se presser. Bleu. Le dernier galet touche la pierre. Le chemin est arrivé. L'escargot est là ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau chante dans l'arbre. J'ai entendu, depuis la cuisine. Vous avez fait un chemin ? Jusqu'à l'escargot. Il est encore sur sa pierre ? Oui, papa. Raphaël a regardé d'abord. Nina a répété la règle. Tu as fini de ranger, Nina ? Oui, maman. Nina donne la main. Raphaël donne l'autre main. Les chaussures laissent des traces mouillées. La gouttière chante plus bas, maintenant. Les galets sont froids. Ils vont sécher. Le seau a encore sa mousse. L'escargot n'a presque pas bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Un oiseau chante dans l'arbre. J'ai entendu. Tu as entendu l'oiseau ? Oui, papa. Tout haut. Nina veut arriver, d'un coup. Elle prend trois galets trop vite. Un galet roule vers la pierre. Ça tombe ! L'&lt;emphasis level="moderate"&gt;éclat de galet&lt;/emphasis&gt; n'est plus là. Il est parti. Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde les galets, un à un. Elle écoute le jardin, un instant. Comme tout à l'heure ? Tu le vois, toi ? Non, plus sur le gris. Nina cherche près de la pierre. Il est là. Sur ce bleu ? Oui, sur ce galet. Elle pose le bleu, sans se presser. Bleu. Le dernier galet touche la pierre. Le chemin est arrivé. L'escargot est là ? Oui, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range les galets. Sami donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>&lt;low-pitch&gt;Un oiseau chante dans l'arbre. J'ai entendu. Tu as entendu l'oiseau ? Oui, papa. Tout haut. Nina veut arriver, d'un coup. Elle prend trois galets trop vite. Un galet roule vers la pierre. Ça tombe ! L'&lt;emphasis&gt;éclat de galet&lt;/emphasis&gt; n'est plus là. Il est parti. Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde les galets, un à un. Elle écoute le jardin, un instant. Comme tout à l'heure ? Tu le vois, toi ? Non, plus sur le gris. Nina cherche près de la pierre. Il est là. Sur ce bleu ? Oui, sur ce galet. Elle pose le bleu, sans se presser. Bleu. Le dernier galet touche la pierre. Le chemin est arrivé. L'escargot est là ? Oui, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1829,7 +1871,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1837,22 +1879,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1863,30 +1909,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de galet</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1895,46 +1941,63 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Un oiseau chante dans l'arbre.
-papa|J'ai entendu, depuis la cuisine.
-papa|Vous avez fait un chemin ?
-enfant-f|Jusqu'à l'escargot.
-papa|Il est encore sur sa pierre ?
+enfant-f|J'ai entendu.
+papa|Tu as entendu l'oiseau ?
 enfant-f|Oui, papa.
-maman|Raphaël a regardé d'abord.
-papa|Nina a répété la règle.
-maman|Tu as fini de ranger, Nina ?
-enfant-f|Oui, maman.
-narrateur|Nina donne la main.
-narrateur|Raphaël donne l'autre main.
-narrateur|Les chaussures laissent des traces mouillées.
-narrateur|La gouttière chante plus bas, maintenant.
-enfant-f|Les galets sont froids.
-papa|Ils vont sécher.
-maman|Le seau a encore sa mousse.
-narrateur|L'escargot n'a presque pas bougé.</t>
+enfant-f|Tout haut.
+narrateur|Nina veut arriver, d'un coup.
+narrateur|Elle prend trois galets trop vite.
+narrateur|Un galet roule vers la pierre.
+enfant-f|Ça tombe !
+narrateur|L'éclat de galet n'est plus là.
+enfant-f|Il est parti.
+narrateur|Nina veut foncer, d'un coup.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde les galets, un à un.
+narrateur|Elle écoute le jardin, un instant.
+enfant-f|Comme tout à l'heure ?
+papa|Tu le vois, toi ?
+enfant-f|Non, plus sur le gris.
+narrateur|Nina cherche près de la pierre.
+enfant-f|Il est là.
+papa|Sur ce bleu ?
+enfant-f|Oui, sur ce galet.
+narrateur|Elle pose le bleu, sans se presser.
+enfant-f|Bleu.
+narrateur|Le dernier galet touche la pierre.
+enfant-f|Le chemin est arrivé.
+maman|L'escargot est là ?
+enfant-f|Oui, maman.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>oiseau,pas</t>
+          <t>oiseau,galets</t>
         </is>
       </c>
     </row>
@@ -1961,17 +2024,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le chemin brille encore un peu. L'escargot reste sur sa pierre. Bonne fin de journée, Nina. Le seau chante tout fin.</t>
+          <t>Le chemin brille un peu, dans la terre. L'escargot reste sur sa pierre. L'éclat est là, papa. Tu le vois sur le galet ? Oui, papa. On est bien, ici. Les chaussures laissent des traces mouillées. Elles vont sécher. Les galets sont froids. Ils vont sécher, eux aussi. Nina pose la joue près du banc. Le bois est sombre, un peu froid. C'est froid. La feuille est là, Nina. Oui, maman. Un oiseau se tait, dans l'arbre. L'éclat de galet tient sur le bleu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le chemin brille encore un peu. L'escargot reste sur sa pierre. Bonne fin de journée, Nina. Le seau chante tout fin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le chemin brille un peu, dans la terre. L'escargot reste sur sa pierre. L'éclat est là, papa. Tu le vois sur le galet ? Oui, papa. On est bien, ici. Les chaussures laissent des traces mouillées. Elles vont sécher. Les galets sont froids. Ils vont sécher, eux aussi. Nina pose la joue près du banc. Le bois est sombre, un peu froid. C'est froid. La feuille est là, Nina. Oui, maman. Un oiseau se tait, dans l'arbre. L'&lt;emphasis level="moderate"&gt;éclat de galet&lt;/emphasis&gt; tient sur le bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le chemin brille un peu, dans la terre. L'escargot reste sur sa pierre. L'éclat est là, papa. Tu le vois sur le galet ? Oui, papa. On est bien, ici. Les chaussures laissent des traces mouillées. Elles vont sécher. Les galets sont froids. Ils vont sécher, eux aussi. Nina pose la joue près du banc. Le bois est sombre, un peu froid. C'est froid. La feuille est là, Nina. Oui, maman. Un oiseau se tait, dans l'arbre. L'&lt;emphasis&gt;éclat de galet&lt;/emphasis&gt; tient sur le bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2018,18 +2081,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2038,12 +2101,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2052,17 +2115,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de galet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2071,11 +2138,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2084,27 +2151,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bleu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le chemin brille encore un peu.
+          <t>narrateur|Le chemin brille un peu, dans la terre.
 narrateur|L'escargot reste sur sa pierre.
-maman|Bonne fin de journée, Nina.
-papa|Le seau chante tout fin.</t>
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur le galet ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|Les chaussures laissent des traces mouillées.
+papa|Elles vont sécher.
+enfant-f|Les galets sont froids.
+maman|Ils vont sécher, eux aussi.
+narrateur|Nina pose la joue près du banc.
+narrateur|Le bois est sombre, un peu froid.
+enfant-f|C'est froid.
+maman|La feuille est là, Nina.
+enfant-f|Oui, maman.
+narrateur|Un oiseau se tait, dans l'arbre.
+narrateur|L'éclat de galet tient sur le bleu.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>jardin</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2210,6 +2299,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>